<commit_message>
feature:- mega event changes and file issue fix
</commit_message>
<xml_diff>
--- a/resources/Create_MegaEvent_Beta.xlsx
+++ b/resources/Create_MegaEvent_Beta.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="ELP_Users" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="MegaEvents" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,11 +413,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:A2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
+        <is>
+          <t>Event Name</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
         <is>
           <t>EventName</t>
         </is>

</xml_diff>